<commit_message>
Verify MySQL integration, sync Power BI filters and strengthen planner input checks
</commit_message>
<xml_diff>
--- a/excel/FreshRoute_Planner.xlsx
+++ b/excel/FreshRoute_Planner.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Planner" sheetId="1" r:id="Re62976a8168d4a85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="2" r:id="Rf3481444db9141cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quotes" sheetId="3" r:id="R2f357022e07e40ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routes" sheetId="4" r:id="R4b057ce14675475b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Planner" sheetId="1" r:id="R92e3c2b478e8402e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="2" r:id="Rd315af5657114ec9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quotes" sheetId="3" r:id="Rdc86bc7d84284974"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routes" sheetId="4" r:id="R04ff1a5086bf4926"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -366,7 +366,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rce173de10d454c99"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R13bee103cb294d70"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -972,19 +972,19 @@
         <x:v>0.69</x:v>
       </x:c>
       <x:c r="E16" s="17" t="n">
-        <x:f>IF(COUNTBLANK(Routes!C7)+COUNTBLANK($C$10)&gt;0,"n.a.",Routes!C7+$C$10)</x:f>
+        <x:f>IF(COUNT(Routes!C7,$C$10)&lt;&gt;2,"n.a.",Routes!C7+$C$10)</x:f>
         <x:v>0.06</x:v>
       </x:c>
       <x:c r="F16" s="18" t="n">
-        <x:f>IF(COUNTBLANK(Routes!D7)+COUNTBLANK($C$11)&gt;0,"n.a.",Routes!D7+$C$11)</x:f>
+        <x:f>IF(COUNT(Routes!D7,$C$11)&lt;&gt;2,"n.a.",Routes!D7+$C$11)</x:f>
         <x:v>0.03</x:v>
       </x:c>
       <x:c r="G16" s="19" t="n">
-        <x:f>IF(COUNTBLANK(Routes!E7)&gt;0,"n.a.",Routes!E7)</x:f>
+        <x:f>IF(COUNT(Routes!E7)&lt;&gt;1,"n.a.",Routes!E7)</x:f>
         <x:v>12000</x:v>
       </x:c>
       <x:c r="H16" s="19" t="str">
-        <x:f>IF(OR(C16&lt;&gt;1,COUNTBLANK($C$6:$C$11)&gt;0,NOT(ISNUMBER(E16)),NOT(ISNUMBER(F16)),NOT(ISNUMBER(G16))),"Unavailable",IF(OR($C$8&lt;=0,$C$9&lt;0,E16&lt;0,F16&lt;0,F16&gt;=1,G16&lt;=0),"Invalid",IF($C$8&lt;=G16,"Yes","Over capacity")))</x:f>
+        <x:f>IF(OR(C16&lt;&gt;1,COUNT($C$6:$C$11)&lt;&gt;6,NOT(ISNUMBER(E16)),NOT(ISNUMBER(F16)),NOT(ISNUMBER(G16))),"Unavailable",IF(OR($C$8&lt;=0,$C$9&lt;0,E16&lt;0,F16&lt;0,F16&gt;=1,G16&lt;=0),"Invalid",IF($C$8&lt;=G16,"Yes","Over capacity")))</x:f>
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="I16" s="19" t="n">
@@ -1028,19 +1028,19 @@
         <x:v>0.56</x:v>
       </x:c>
       <x:c r="E17" s="17" t="n">
-        <x:f>IF(COUNTBLANK(Routes!C8)+COUNTBLANK($C$10)&gt;0,"n.a.",Routes!C8+$C$10)</x:f>
+        <x:f>IF(COUNT(Routes!C8,$C$10)&lt;&gt;2,"n.a.",Routes!C8+$C$10)</x:f>
         <x:v>0.19</x:v>
       </x:c>
       <x:c r="F17" s="18" t="n">
-        <x:f>IF(COUNTBLANK(Routes!D8)+COUNTBLANK($C$11)&gt;0,"n.a.",Routes!D8+$C$11)</x:f>
+        <x:f>IF(COUNT(Routes!D8,$C$11)&lt;&gt;2,"n.a.",Routes!D8+$C$11)</x:f>
         <x:v>0.06</x:v>
       </x:c>
       <x:c r="G17" s="19" t="n">
-        <x:f>IF(COUNTBLANK(Routes!E8)&gt;0,"n.a.",Routes!E8)</x:f>
+        <x:f>IF(COUNT(Routes!E8)&lt;&gt;1,"n.a.",Routes!E8)</x:f>
         <x:v>16000</x:v>
       </x:c>
       <x:c r="H17" s="19" t="str">
-        <x:f>IF(OR(C17&lt;&gt;1,COUNTBLANK($C$6:$C$11)&gt;0,NOT(ISNUMBER(E17)),NOT(ISNUMBER(F17)),NOT(ISNUMBER(G17))),"Unavailable",IF(OR($C$8&lt;=0,$C$9&lt;0,E17&lt;0,F17&lt;0,F17&gt;=1,G17&lt;=0),"Invalid",IF($C$8&lt;=G17,"Yes","Over capacity")))</x:f>
+        <x:f>IF(OR(C17&lt;&gt;1,COUNT($C$6:$C$11)&lt;&gt;6,NOT(ISNUMBER(E17)),NOT(ISNUMBER(F17)),NOT(ISNUMBER(G17))),"Unavailable",IF(OR($C$8&lt;=0,$C$9&lt;0,E17&lt;0,F17&lt;0,F17&gt;=1,G17&lt;=0),"Invalid",IF($C$8&lt;=G17,"Yes","Over capacity")))</x:f>
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="I17" s="19" t="n">
@@ -1084,19 +1084,19 @@
         <x:v>n.a.</x:v>
       </x:c>
       <x:c r="E18" s="17" t="n">
-        <x:f>IF(COUNTBLANK(Routes!C9)+COUNTBLANK($C$10)&gt;0,"n.a.",Routes!C9+$C$10)</x:f>
+        <x:f>IF(COUNT(Routes!C9,$C$10)&lt;&gt;2,"n.a.",Routes!C9+$C$10)</x:f>
         <x:v>0.04</x:v>
       </x:c>
       <x:c r="F18" s="18" t="n">
-        <x:f>IF(COUNTBLANK(Routes!D9)+COUNTBLANK($C$11)&gt;0,"n.a.",Routes!D9+$C$11)</x:f>
+        <x:f>IF(COUNT(Routes!D9,$C$11)&lt;&gt;2,"n.a.",Routes!D9+$C$11)</x:f>
         <x:v>0.025</x:v>
       </x:c>
       <x:c r="G18" s="19" t="n">
-        <x:f>IF(COUNTBLANK(Routes!E9)&gt;0,"n.a.",Routes!E9)</x:f>
+        <x:f>IF(COUNT(Routes!E9)&lt;&gt;1,"n.a.",Routes!E9)</x:f>
         <x:v>10000</x:v>
       </x:c>
       <x:c r="H18" s="19" t="str">
-        <x:f>IF(OR(C18&lt;&gt;1,COUNTBLANK($C$6:$C$11)&gt;0,NOT(ISNUMBER(E18)),NOT(ISNUMBER(F18)),NOT(ISNUMBER(G18))),"Unavailable",IF(OR($C$8&lt;=0,$C$9&lt;0,E18&lt;0,F18&lt;0,F18&gt;=1,G18&lt;=0),"Invalid",IF($C$8&lt;=G18,"Yes","Over capacity")))</x:f>
+        <x:f>IF(OR(C18&lt;&gt;1,COUNT($C$6:$C$11)&lt;&gt;6,NOT(ISNUMBER(E18)),NOT(ISNUMBER(F18)),NOT(ISNUMBER(G18))),"Unavailable",IF(OR($C$8&lt;=0,$C$9&lt;0,E18&lt;0,F18&lt;0,F18&gt;=1,G18&lt;=0),"Invalid",IF($C$8&lt;=G18,"Yes","Over capacity")))</x:f>
         <x:v>Unavailable</x:v>
       </x:c>
       <x:c r="I18" s="19" t="str">
@@ -1777,7 +1777,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0158847146f74296"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9cb8fefccfd4ea0"/>
 </x:worksheet>
 </file>
 
@@ -4207,7 +4207,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99cfb1c3b9e7413d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra509f13fe54d4a52"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5203,7 +5203,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc2b0f8dc1d44752"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2197ac025ba94da0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>